<commit_message>
Fix some bug in CTable::DrawImage
</commit_message>
<xml_diff>
--- a/Experts/Anhnt/Document/MQL5 Note/TableDesign.xlsx
+++ b/Experts/Anhnt/Document/MQL5 Note/TableDesign.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nguye\AppData\Roaming\MetaQuotes\Terminal\D0E8209F77C8CF37AD8BF550E51FF075\MQL5\Experts\Anhnt\Document\MQL5 Note\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B970B588-F0B1-4481-A54B-22048180D00C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F3CF7AA-BF2D-45F6-9CDC-6377DC35CDDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Realtime" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="3" r:id="rId2"/>
-    <sheet name="Sheet1" sheetId="2" r:id="rId3"/>
+    <sheet name="Trailling" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="27">
   <si>
     <t>Symbol</t>
   </si>
@@ -113,6 +113,12 @@
   </si>
   <si>
     <t>Pip (Percentage in Point)</t>
+  </si>
+  <si>
+    <t>RiskRate</t>
+  </si>
+  <si>
+    <t>Note</t>
   </si>
 </sst>
 </file>
@@ -636,9 +642,18 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8DD6A09-4844-4E7E-876D-C6871822B0CD}">
-  <dimension ref="A1"/>
+  <dimension ref="B1:C1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>